<commit_message>
several changes and cleaning
</commit_message>
<xml_diff>
--- a/logs/experiments_not_systematic/experiments_mapping_order_encoding/experiments_mapping_order_encoding.xlsx
+++ b/logs/experiments_not_systematic/experiments_mapping_order_encoding/experiments_mapping_order_encoding.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mgep-my.sharepoint.com/personal/uxue_ballarin_alumni_mondragon_edu/Documents/Semestre 8-Erasmus/Simula/ship_qnn/logs/experiments_not_systematic/experiments_mapping_order_encoding/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="105" documentId="11_AD4D2F04E46CFB4ACB3E20D455D6CCDA693EDF1F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0B6A5BE-9FAE-4E34-9C36-470939D1ABDF}"/>
+  <xr:revisionPtr revIDLastSave="109" documentId="11_AD4D2F04E46CFB4ACB3E20D455D6CCDA693EDF1F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D3ABFBA-A81B-4DEF-9D43-11B0D25084DA}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5580" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <calcPr calcId="162913"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId3"/>
+    <pivotCache cacheId="19" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2380" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2374" uniqueCount="293">
   <si>
     <t>date</t>
   </si>
@@ -12870,7 +12870,291 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B7F402C0-60A3-4F37-9EFD-E8650E226302}" name="TablaDinámica2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{85510CF5-2A69-4AE5-9829-C84B5FC72F1C}" name="TablaDinámica1" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:L34" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="75">
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="9">
+        <item x="0"/>
+        <item h="1" sd="0" x="7"/>
+        <item h="1" sd="0" x="3"/>
+        <item h="1" sd="0" x="5"/>
+        <item h="1" sd="0" x="4"/>
+        <item h="1" sd="0" x="6"/>
+        <item h="1" sd="0" x="1"/>
+        <item h="1" sd="0" x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+  </pivotFields>
+  <rowFields count="4">
+    <field x="18"/>
+    <field x="21"/>
+    <field x="22"/>
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="31">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="2">
+      <x/>
+    </i>
+    <i r="3">
+      <x/>
+    </i>
+    <i r="3">
+      <x v="1"/>
+    </i>
+    <i r="3">
+      <x v="2"/>
+    </i>
+    <i r="3">
+      <x v="3"/>
+    </i>
+    <i r="3">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="2">
+      <x/>
+    </i>
+    <i r="3">
+      <x/>
+    </i>
+    <i r="3">
+      <x v="1"/>
+    </i>
+    <i r="3">
+      <x v="2"/>
+    </i>
+    <i r="3">
+      <x v="3"/>
+    </i>
+    <i r="3">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="2">
+      <x/>
+    </i>
+    <i r="3">
+      <x/>
+    </i>
+    <i r="3">
+      <x v="1"/>
+    </i>
+    <i r="3">
+      <x v="2"/>
+    </i>
+    <i r="3">
+      <x v="3"/>
+    </i>
+    <i r="3">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="11">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+    <i i="3">
+      <x v="3"/>
+    </i>
+    <i i="4">
+      <x v="4"/>
+    </i>
+    <i i="5">
+      <x v="5"/>
+    </i>
+    <i i="6">
+      <x v="6"/>
+    </i>
+    <i i="7">
+      <x v="7"/>
+    </i>
+    <i i="8">
+      <x v="8"/>
+    </i>
+    <i i="9">
+      <x v="9"/>
+    </i>
+    <i i="10">
+      <x v="10"/>
+    </i>
+  </colItems>
+  <dataFields count="11">
+    <dataField name="Promedio de Val Global Open R2" fld="36" subtotal="average" baseField="22" baseItem="0"/>
+    <dataField name="Promedio de Val Global Closed R2" fld="37" subtotal="average" baseField="22" baseItem="0"/>
+    <dataField name="Promedio de Surge Velocity Global open R2" fld="51" subtotal="average" baseField="22" baseItem="0"/>
+    <dataField name="Promedio de Sway Velocity Global open R2" fld="58" subtotal="average" baseField="22" baseItem="0"/>
+    <dataField name="Promedio de Yaw Rate Global open R2" fld="65" subtotal="average" baseField="22" baseItem="0"/>
+    <dataField name="Promedio de Yaw Angle Global open R2" fld="72" subtotal="average" baseField="22" baseItem="0"/>
+    <dataField name="Promedio de Surge Velocity Global closed R2" fld="53" subtotal="average" baseField="22" baseItem="5"/>
+    <dataField name="Promedio de Sway Velocity Global closed R2" fld="60" subtotal="average" baseField="22" baseItem="5"/>
+    <dataField name="Promedio de Yaw Rate Global closed R2" fld="67" subtotal="average" baseField="22" baseItem="5"/>
+    <dataField name="Promedio de Yaw Angle Global closed R2" fld="74" subtotal="average" baseField="22" baseItem="5"/>
+    <dataField name="Cuenta de model_id" fld="1" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B7F402C0-60A3-4F37-9EFD-E8650E226302}" name="TablaDinámica2" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="O3:P34" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="75">
     <pivotField numFmtId="164" showAll="0"/>
@@ -13090,398 +13374,6 @@
   </colItems>
   <dataFields count="1">
     <dataField name="Promedio de global open R2" fld="42" subtotal="average" baseField="22" baseItem="7"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{85510CF5-2A69-4AE5-9829-C84B5FC72F1C}" name="TablaDinámica1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:L70" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="75">
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="9">
-        <item x="0"/>
-        <item h="1" sd="0" x="7"/>
-        <item h="1" sd="0" x="3"/>
-        <item h="1" sd="0" x="5"/>
-        <item h="1" sd="0" x="4"/>
-        <item h="1" sd="0" x="6"/>
-        <item h="1" sd="0" x="1"/>
-        <item h="1" sd="0" x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-  </pivotFields>
-  <rowFields count="4">
-    <field x="18"/>
-    <field x="21"/>
-    <field x="22"/>
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="67">
-    <i>
-      <x/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="2">
-      <x/>
-    </i>
-    <i r="3">
-      <x/>
-    </i>
-    <i r="3">
-      <x v="1"/>
-    </i>
-    <i r="3">
-      <x v="2"/>
-    </i>
-    <i r="3">
-      <x v="3"/>
-    </i>
-    <i r="3">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="2">
-      <x/>
-    </i>
-    <i r="3">
-      <x/>
-    </i>
-    <i r="3">
-      <x v="1"/>
-    </i>
-    <i r="3">
-      <x v="2"/>
-    </i>
-    <i r="3">
-      <x v="3"/>
-    </i>
-    <i r="3">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="2">
-      <x/>
-    </i>
-    <i r="3">
-      <x/>
-    </i>
-    <i r="3">
-      <x v="1"/>
-    </i>
-    <i r="3">
-      <x v="2"/>
-    </i>
-    <i r="3">
-      <x v="3"/>
-    </i>
-    <i r="3">
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="2">
-      <x/>
-    </i>
-    <i r="3">
-      <x/>
-    </i>
-    <i r="3">
-      <x v="1"/>
-    </i>
-    <i r="3">
-      <x v="2"/>
-    </i>
-    <i r="3">
-      <x v="3"/>
-    </i>
-    <i r="3">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="2">
-      <x/>
-    </i>
-    <i r="3">
-      <x/>
-    </i>
-    <i r="3">
-      <x v="1"/>
-    </i>
-    <i r="3">
-      <x v="2"/>
-    </i>
-    <i r="3">
-      <x v="3"/>
-    </i>
-    <i r="3">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="2">
-      <x/>
-    </i>
-    <i r="3">
-      <x/>
-    </i>
-    <i r="3">
-      <x v="1"/>
-    </i>
-    <i r="3">
-      <x v="2"/>
-    </i>
-    <i r="3">
-      <x v="3"/>
-    </i>
-    <i r="3">
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="2">
-      <x/>
-    </i>
-    <i r="3">
-      <x/>
-    </i>
-    <i r="3">
-      <x v="1"/>
-    </i>
-    <i r="3">
-      <x v="2"/>
-    </i>
-    <i r="3">
-      <x v="3"/>
-    </i>
-    <i r="3">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="2">
-      <x/>
-    </i>
-    <i r="3">
-      <x/>
-    </i>
-    <i r="3">
-      <x v="1"/>
-    </i>
-    <i r="3">
-      <x v="2"/>
-    </i>
-    <i r="3">
-      <x v="3"/>
-    </i>
-    <i r="3">
-      <x v="4"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="2">
-      <x/>
-    </i>
-    <i r="3">
-      <x/>
-    </i>
-    <i r="3">
-      <x v="1"/>
-    </i>
-    <i r="3">
-      <x v="2"/>
-    </i>
-    <i r="3">
-      <x v="3"/>
-    </i>
-    <i r="3">
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="11">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-    <i i="2">
-      <x v="2"/>
-    </i>
-    <i i="3">
-      <x v="3"/>
-    </i>
-    <i i="4">
-      <x v="4"/>
-    </i>
-    <i i="5">
-      <x v="5"/>
-    </i>
-    <i i="6">
-      <x v="6"/>
-    </i>
-    <i i="7">
-      <x v="7"/>
-    </i>
-    <i i="8">
-      <x v="8"/>
-    </i>
-    <i i="9">
-      <x v="9"/>
-    </i>
-    <i i="10">
-      <x v="10"/>
-    </i>
-  </colItems>
-  <dataFields count="11">
-    <dataField name="Promedio de Val Global Open R2" fld="36" subtotal="average" baseField="22" baseItem="0"/>
-    <dataField name="Promedio de Val Global Closed R2" fld="37" subtotal="average" baseField="22" baseItem="0"/>
-    <dataField name="Promedio de Surge Velocity Global open R2" fld="51" subtotal="average" baseField="22" baseItem="0"/>
-    <dataField name="Promedio de Sway Velocity Global open R2" fld="58" subtotal="average" baseField="22" baseItem="0"/>
-    <dataField name="Promedio de Yaw Rate Global open R2" fld="65" subtotal="average" baseField="22" baseItem="0"/>
-    <dataField name="Promedio de Yaw Angle Global open R2" fld="72" subtotal="average" baseField="22" baseItem="0"/>
-    <dataField name="Promedio de Surge Velocity Global closed R2" fld="53" subtotal="average" baseField="22" baseItem="5"/>
-    <dataField name="Promedio de Sway Velocity Global closed R2" fld="60" subtotal="average" baseField="22" baseItem="5"/>
-    <dataField name="Promedio de Yaw Rate Global closed R2" fld="67" subtotal="average" baseField="22" baseItem="5"/>
-    <dataField name="Promedio de Yaw Angle Global closed R2" fld="74" subtotal="average" baseField="22" baseItem="5"/>
-    <dataField name="Cuenta de model_id" fld="1" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -47731,21 +47623,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F26549A3-A0B3-440A-B21C-C30F36E0E432}">
-  <dimension ref="A3:P70"/>
+  <dimension ref="A3:P34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="38.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="34.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="35.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="39.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="39.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="35.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="36.21875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="34.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="38.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="38.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="34.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="19.88671875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="25.44140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -48191,38 +48083,38 @@
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
-        <v>86</v>
+      <c r="A13" s="5">
+        <v>5</v>
       </c>
       <c r="B13" s="8">
-        <v>0.29506068470817776</v>
+        <v>0.20750537952444273</v>
       </c>
       <c r="C13" s="8">
-        <v>-0.12378029829383955</v>
+        <v>-5.5444678591765315E-2</v>
       </c>
       <c r="D13" s="8">
-        <v>0.1142253070461127</v>
+        <v>-4.1485316126547288E-2</v>
       </c>
       <c r="E13" s="8">
-        <v>0.37179522710706953</v>
+        <v>0.29983358906334079</v>
       </c>
       <c r="F13" s="8">
-        <v>0.45280514962614282</v>
+        <v>0.32799067349390632</v>
       </c>
       <c r="G13" s="8">
-        <v>0.1069354202279541</v>
+        <v>0.26197170552156823</v>
       </c>
       <c r="H13" s="8">
-        <v>-1.9830317565831646E-2</v>
+        <v>-0.10204935041200761</v>
       </c>
       <c r="I13" s="8">
-        <v>-0.10069634426988509</v>
+        <v>-1.2450701636136218E-2</v>
       </c>
       <c r="J13" s="8">
-        <v>-0.17080468211179936</v>
+        <v>-1.8926023619588152E-2</v>
       </c>
       <c r="K13" s="8">
-        <v>-5.2337127140523507E-2</v>
+        <v>-5.1580733889718601E-2</v>
       </c>
       <c r="L13" s="8">
         <v>5</v>
@@ -48235,41 +48127,41 @@
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A14" s="7">
-        <v>0</v>
+      <c r="A14" s="4" t="s">
+        <v>94</v>
       </c>
       <c r="B14" s="8">
-        <v>0.34431591735198419</v>
+        <v>0.40782266884150087</v>
       </c>
       <c r="C14" s="8">
-        <v>-0.30180681135839349</v>
+        <v>-0.11205067450956041</v>
       </c>
       <c r="D14" s="8">
-        <v>6.5600054680017061E-2</v>
+        <v>0.15491957209600865</v>
       </c>
       <c r="E14" s="8">
-        <v>0.45915318594561838</v>
+        <v>0.40941404869619208</v>
       </c>
       <c r="F14" s="8">
-        <v>0.52249150983550952</v>
+        <v>0.2561382429608805</v>
       </c>
       <c r="G14" s="8">
-        <v>0.15601827248508801</v>
+        <v>0.68642496195515867</v>
       </c>
       <c r="H14" s="8">
-        <v>-9.2873044621338385E-2</v>
+        <v>-5.4366388195809696E-2</v>
       </c>
       <c r="I14" s="8">
-        <v>-0.27016345014442372</v>
+        <v>-0.1152566860974933</v>
       </c>
       <c r="J14" s="8">
-        <v>-0.36040153532500158</v>
+        <v>4.8335791804963793E-2</v>
       </c>
       <c r="K14" s="8">
-        <v>-1.979349430102717E-2</v>
+        <v>-0.38007554271296284</v>
       </c>
       <c r="L14" s="8">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="O14" s="4" t="s">
         <v>94</v>
@@ -48279,41 +48171,41 @@
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A15" s="7">
+      <c r="A15" s="5">
         <v>1</v>
       </c>
       <c r="B15" s="8">
-        <v>0.28485631377620241</v>
+        <v>0.40307212927502833</v>
       </c>
       <c r="C15" s="8">
-        <v>-4.1805110202016438E-2</v>
+        <v>-0.38409278654220974</v>
       </c>
       <c r="D15" s="8">
-        <v>8.547142143567199E-2</v>
+        <v>0.24286635287172137</v>
       </c>
       <c r="E15" s="8">
-        <v>0.36355314659782179</v>
+        <v>0.36088554712190801</v>
       </c>
       <c r="F15" s="8">
-        <v>0.43674849960814949</v>
+        <v>0.11767541403108975</v>
       </c>
       <c r="G15" s="8">
-        <v>7.9046545046571715E-2</v>
+        <v>0.78819312824362509</v>
       </c>
       <c r="H15" s="8">
-        <v>3.6025595591620219E-2</v>
+        <v>-3.4457935648817717E-2</v>
       </c>
       <c r="I15" s="8">
-        <v>-2.522338591774553E-2</v>
+        <v>-0.47559922109553432</v>
       </c>
       <c r="J15" s="8">
-        <v>-0.12848071824646801</v>
+        <v>-0.1390336640222814</v>
       </c>
       <c r="K15" s="8">
-        <v>-0.1080307453615514</v>
+        <v>-0.94611270969677663</v>
       </c>
       <c r="L15" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O15" s="5">
         <v>3</v>
@@ -48323,41 +48215,41 @@
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A16" s="7">
-        <v>2</v>
+      <c r="A16" s="6" t="s">
+        <v>86</v>
       </c>
       <c r="B16" s="8">
-        <v>0.2311023127493198</v>
+        <v>0.40307212927502833</v>
       </c>
       <c r="C16" s="8">
-        <v>-0.1178759687047672</v>
+        <v>-0.38409278654220974</v>
       </c>
       <c r="D16" s="8">
-        <v>0.1680536295971051</v>
+        <v>0.24286635287172137</v>
       </c>
       <c r="E16" s="8">
-        <v>0.30458926407374493</v>
+        <v>0.36088554712190801</v>
       </c>
       <c r="F16" s="8">
-        <v>0.42350627147833309</v>
+        <v>0.11767541403108975</v>
       </c>
       <c r="G16" s="8">
-        <v>2.9708434543163079E-2</v>
+        <v>0.78819312824362509</v>
       </c>
       <c r="H16" s="8">
-        <v>4.8565361337225887E-2</v>
+        <v>-3.4457935648817717E-2</v>
       </c>
       <c r="I16" s="8">
-        <v>-0.16301175281928121</v>
+        <v>-0.47559922109553432</v>
       </c>
       <c r="J16" s="8">
-        <v>-0.18960765059669149</v>
+        <v>-0.1390336640222814</v>
       </c>
       <c r="K16" s="8">
-        <v>-3.2830780843827512E-2</v>
+        <v>-0.94611270969677663</v>
       </c>
       <c r="L16" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O16" s="6" t="s">
         <v>86</v>
@@ -48368,37 +48260,37 @@
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" s="7">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B17" s="8">
-        <v>0.29139493490452029</v>
+        <v>0.4265670805307275</v>
       </c>
       <c r="C17" s="8">
-        <v>-2.469090820575515E-2</v>
+        <v>-0.56800594377510771</v>
       </c>
       <c r="D17" s="8">
-        <v>0.1403375643947061</v>
+        <v>0.26567018161996392</v>
       </c>
       <c r="E17" s="8">
-        <v>0.38213698141119729</v>
+        <v>0.39542136922712878</v>
       </c>
       <c r="F17" s="8">
-        <v>0.43798381713474788</v>
+        <v>0.14489457713923379</v>
       </c>
       <c r="G17" s="8">
-        <v>5.2883380232705779E-2</v>
+        <v>0.80326104224981365</v>
       </c>
       <c r="H17" s="8">
-        <v>-3.057234965817246E-2</v>
+        <v>-0.30697220600760572</v>
       </c>
       <c r="I17" s="8">
-        <v>5.1081954399951668E-2</v>
+        <v>-0.68315349377639945</v>
       </c>
       <c r="J17" s="8">
-        <v>6.5432350582657062E-3</v>
+        <v>-0.19170100301661019</v>
       </c>
       <c r="K17" s="8">
-        <v>-5.6153181355659942E-2</v>
+        <v>-1.3208823454805869</v>
       </c>
       <c r="L17" s="8">
         <v>1</v>
@@ -48412,37 +48304,37 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B18" s="8">
-        <v>0.32363394475886198</v>
+        <v>0.34913976236230748</v>
       </c>
       <c r="C18" s="8">
-        <v>-0.13272269299826539</v>
+        <v>-0.14319329478432299</v>
       </c>
       <c r="D18" s="8">
-        <v>0.1116638651230631</v>
+        <v>0.16876904308305879</v>
       </c>
       <c r="E18" s="8">
-        <v>0.34954355750696531</v>
+        <v>0.30962560357124702</v>
       </c>
       <c r="F18" s="8">
-        <v>0.44329565007397398</v>
+        <v>8.0092309452948429E-2</v>
       </c>
       <c r="G18" s="8">
-        <v>0.21702046883224191</v>
+        <v>0.7780452519197949</v>
       </c>
       <c r="H18" s="8">
-        <v>-6.0297150478493489E-2</v>
+        <v>0.17272212982402871</v>
       </c>
       <c r="I18" s="8">
-        <v>-9.6165086867926686E-2</v>
+        <v>-0.2309835712801058</v>
       </c>
       <c r="J18" s="8">
-        <v>-0.18207674144910141</v>
+        <v>-6.0824068280210142E-2</v>
       </c>
       <c r="K18" s="8">
-        <v>-4.4877433840551539E-2</v>
+        <v>-0.55245686129743032</v>
       </c>
       <c r="L18" s="8">
         <v>1</v>
@@ -48455,41 +48347,41 @@
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A19" s="5">
-        <v>5</v>
+      <c r="A19" s="7">
+        <v>2</v>
       </c>
       <c r="B19" s="8">
-        <v>0.20750537952444273</v>
+        <v>0.40270321163788242</v>
       </c>
       <c r="C19" s="8">
-        <v>-5.5444678591765315E-2</v>
+        <v>-0.36173987753704911</v>
       </c>
       <c r="D19" s="8">
-        <v>-4.1485316126547288E-2</v>
+        <v>0.24474388669368799</v>
       </c>
       <c r="E19" s="8">
-        <v>0.29983358906334079</v>
+        <v>0.35186930212477052</v>
       </c>
       <c r="F19" s="8">
-        <v>0.32799067349390632</v>
+        <v>0.1252465789378607</v>
       </c>
       <c r="G19" s="8">
-        <v>0.26197170552156823</v>
+        <v>0.78029832059154924</v>
       </c>
       <c r="H19" s="8">
-        <v>-0.10204935041200761</v>
+        <v>-0.15506311711034779</v>
       </c>
       <c r="I19" s="8">
-        <v>-1.2450701636136218E-2</v>
+        <v>-0.34010410849117578</v>
       </c>
       <c r="J19" s="8">
-        <v>-1.8926023619588152E-2</v>
+        <v>-8.9886049829636328E-2</v>
       </c>
       <c r="K19" s="8">
-        <v>-5.1580733889718601E-2</v>
+        <v>-0.77157729202631997</v>
       </c>
       <c r="L19" s="8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O19" s="6" t="s">
         <v>208</v>
@@ -48499,41 +48391,41 @@
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A20" s="6" t="s">
-        <v>86</v>
+      <c r="A20" s="7">
+        <v>3</v>
       </c>
       <c r="B20" s="8">
-        <v>0.20750537952444273</v>
+        <v>0.41227629571046143</v>
       </c>
       <c r="C20" s="8">
-        <v>-5.5444678591765315E-2</v>
+        <v>-0.35117530143303433</v>
       </c>
       <c r="D20" s="8">
-        <v>-4.1485316126547288E-2</v>
+        <v>0.25532204503223749</v>
       </c>
       <c r="E20" s="8">
-        <v>0.29983358906334079</v>
+        <v>0.35980052369876431</v>
       </c>
       <c r="F20" s="8">
-        <v>0.32799067349390632</v>
+        <v>0.1168874035781555</v>
       </c>
       <c r="G20" s="8">
-        <v>0.26197170552156823</v>
+        <v>0.79105514782979947</v>
       </c>
       <c r="H20" s="8">
-        <v>-0.10204935041200761</v>
+        <v>7.1535294243375125E-2</v>
       </c>
       <c r="I20" s="8">
-        <v>-1.2450701636136218E-2</v>
+        <v>-0.45395816669139721</v>
       </c>
       <c r="J20" s="8">
-        <v>-1.8926023619588152E-2</v>
+        <v>-0.15758815650815319</v>
       </c>
       <c r="K20" s="8">
-        <v>-5.1580733889718601E-2</v>
+        <v>-0.79379475304162295</v>
       </c>
       <c r="L20" s="8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O20" s="6" t="s">
         <v>191</v>
@@ -48544,37 +48436,37 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" s="7">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B21" s="8">
-        <v>0.15967267451546421</v>
+        <v>0.42467429613376301</v>
       </c>
       <c r="C21" s="8">
-        <v>4.9146993484370516E-3</v>
+        <v>-0.49634951518153458</v>
       </c>
       <c r="D21" s="8">
-        <v>-7.9997782776323634E-2</v>
+        <v>0.27982660792965869</v>
       </c>
       <c r="E21" s="8">
-        <v>0.17500399017068599</v>
+        <v>0.38771093698762937</v>
       </c>
       <c r="F21" s="8">
-        <v>0.15716450017593181</v>
+        <v>0.12125620104725029</v>
       </c>
       <c r="G21" s="8">
-        <v>0.28963119975383539</v>
+        <v>0.78830587862716817</v>
       </c>
       <c r="H21" s="8">
-        <v>-9.6274129027351218E-2</v>
+        <v>4.5488220806461088E-2</v>
       </c>
       <c r="I21" s="8">
-        <v>2.183741735599665E-2</v>
+        <v>-0.66979676523859322</v>
       </c>
       <c r="J21" s="8">
-        <v>5.7468015629853257E-2</v>
+        <v>-0.19516904247679709</v>
       </c>
       <c r="K21" s="8">
-        <v>-8.897537303856895E-2</v>
+        <v>-1.2918522966379229</v>
       </c>
       <c r="L21" s="8">
         <v>1</v>
@@ -48587,41 +48479,41 @@
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A22" s="7">
-        <v>1</v>
+      <c r="A22" s="5">
+        <v>3</v>
       </c>
       <c r="B22" s="8">
-        <v>0.24166103175684381</v>
+        <v>0.44214423893222754</v>
       </c>
       <c r="C22" s="8">
-        <v>-0.16716144022542281</v>
+        <v>5.9381069547292865E-2</v>
       </c>
       <c r="D22" s="8">
-        <v>-1.7507094397738902E-2</v>
+        <v>0.10824553380471022</v>
       </c>
       <c r="E22" s="8">
-        <v>0.28367094501474938</v>
+        <v>0.47664456889684359</v>
       </c>
       <c r="F22" s="8">
-        <v>0.28314618367504851</v>
+        <v>0.38540290740041361</v>
       </c>
       <c r="G22" s="8">
-        <v>0.30021052057523961</v>
+        <v>0.66212392028841749</v>
       </c>
       <c r="H22" s="8">
-        <v>-0.1302367667655264</v>
+        <v>-0.11002622203250137</v>
       </c>
       <c r="I22" s="8">
-        <v>-0.14711832778441369</v>
+        <v>0.13499579743245385</v>
       </c>
       <c r="J22" s="8">
-        <v>-0.16021259650711081</v>
+        <v>0.20226114065201303</v>
       </c>
       <c r="K22" s="8">
-        <v>-1.434725805592452E-2</v>
+        <v>-2.0336451665511103E-2</v>
       </c>
       <c r="L22" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O22" s="6" t="s">
         <v>141</v>
@@ -48631,41 +48523,41 @@
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A23" s="7">
-        <v>2</v>
+      <c r="A23" s="5">
+        <v>5</v>
       </c>
       <c r="B23" s="8">
-        <v>0.20535317591330229</v>
+        <v>0.37825163831724673</v>
       </c>
       <c r="C23" s="8">
-        <v>-8.3975510829330913E-2</v>
+        <v>-1.1440306533764349E-2</v>
       </c>
       <c r="D23" s="8">
-        <v>-2.7760069838186349E-2</v>
+        <v>0.11364682961159425</v>
       </c>
       <c r="E23" s="8">
-        <v>0.32178626745410199</v>
+        <v>0.3907120300698248</v>
       </c>
       <c r="F23" s="8">
-        <v>0.37894793526018622</v>
+        <v>0.26533640745113807</v>
       </c>
       <c r="G23" s="8">
-        <v>0.22985338703324931</v>
+        <v>0.60895783733343389</v>
       </c>
       <c r="H23" s="8">
-        <v>-7.1598455885512946E-2</v>
+        <v>-1.8615006906109999E-2</v>
       </c>
       <c r="I23" s="8">
-        <v>-4.5363412860744079E-2</v>
+        <v>-5.1666346293995965E-3</v>
       </c>
       <c r="J23" s="8">
-        <v>-8.0452085009623309E-2</v>
+        <v>8.1779898785159691E-2</v>
       </c>
       <c r="K23" s="8">
-        <v>-8.2563928040926715E-2</v>
+        <v>-0.17377746677660094</v>
       </c>
       <c r="L23" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O23" s="6" t="s">
         <v>158</v>
@@ -48675,41 +48567,41 @@
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A24" s="7">
-        <v>3</v>
+      <c r="A24" s="4" t="s">
+        <v>98</v>
       </c>
       <c r="B24" s="8">
-        <v>0.1951699105167943</v>
+        <v>0.47741928327525696</v>
       </c>
       <c r="C24" s="8">
-        <v>1.7476405162737959E-2</v>
+        <v>-0.42869104043873196</v>
       </c>
       <c r="D24" s="8">
-        <v>-1.734751051608607E-2</v>
+        <v>0.14095666727538431</v>
       </c>
       <c r="E24" s="8">
-        <v>0.29141345073067237</v>
+        <v>0.60372608567093289</v>
       </c>
       <c r="F24" s="8">
-        <v>0.32985594128165979</v>
+        <v>0.57613197232738822</v>
       </c>
       <c r="G24" s="8">
-        <v>0.27608889345485849</v>
+        <v>0.45222243483909075</v>
       </c>
       <c r="H24" s="8">
-        <v>-0.102539133470694</v>
+        <v>-9.0522287863725737E-2</v>
       </c>
       <c r="I24" s="8">
-        <v>9.1267102025854308E-2</v>
+        <v>-0.61972416913221184</v>
       </c>
       <c r="J24" s="8">
-        <v>0.15827455263964471</v>
+        <v>-0.52943744080603383</v>
       </c>
       <c r="K24" s="8">
-        <v>-3.3526792561709318E-2</v>
+        <v>-0.34408027201348812</v>
       </c>
       <c r="L24" s="8">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="O24" s="4" t="s">
         <v>98</v>
@@ -48719,41 +48611,41 @@
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A25" s="7">
-        <v>4</v>
+      <c r="A25" s="5">
+        <v>1</v>
       </c>
       <c r="B25" s="8">
-        <v>0.235670104919809</v>
+        <v>0.65806631564195817</v>
       </c>
       <c r="C25" s="8">
-        <v>-4.8477546415247902E-2</v>
+        <v>-1.0167858250710053</v>
       </c>
       <c r="D25" s="8">
-        <v>-6.4814123104401489E-2</v>
+        <v>0.32384906827838522</v>
       </c>
       <c r="E25" s="8">
-        <v>0.42729329194649429</v>
+        <v>0.76654963396403786</v>
       </c>
       <c r="F25" s="8">
-        <v>0.49083880707670541</v>
+        <v>0.64243870399516623</v>
       </c>
       <c r="G25" s="8">
-        <v>0.21407452679065839</v>
+        <v>0.69546456982198634</v>
       </c>
       <c r="H25" s="8">
-        <v>-0.1095982669109534</v>
+        <v>-5.3763517755991821E-2</v>
       </c>
       <c r="I25" s="8">
-        <v>1.7123713082625721E-2</v>
+        <v>-1.5735104634281676</v>
       </c>
       <c r="J25" s="8">
-        <v>-6.9708004850704608E-2</v>
+        <v>-1.1934464325502776</v>
       </c>
       <c r="K25" s="8">
-        <v>-3.8490317751463499E-2</v>
+        <v>-0.85240190689112227</v>
       </c>
       <c r="L25" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O25" s="5">
         <v>3</v>
@@ -48763,41 +48655,41 @@
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
-        <v>94</v>
+      <c r="A26" s="6" t="s">
+        <v>86</v>
       </c>
       <c r="B26" s="8">
-        <v>0.40782266884150087</v>
+        <v>0.65806631564195817</v>
       </c>
       <c r="C26" s="8">
-        <v>-0.11205067450956041</v>
+        <v>-1.0167858250710053</v>
       </c>
       <c r="D26" s="8">
-        <v>0.15491957209600865</v>
+        <v>0.32384906827838522</v>
       </c>
       <c r="E26" s="8">
-        <v>0.40941404869619208</v>
+        <v>0.76654963396403786</v>
       </c>
       <c r="F26" s="8">
-        <v>0.2561382429608805</v>
+        <v>0.64243870399516623</v>
       </c>
       <c r="G26" s="8">
-        <v>0.68642496195515867</v>
+        <v>0.69546456982198634</v>
       </c>
       <c r="H26" s="8">
-        <v>-5.4366388195809696E-2</v>
+        <v>-5.3763517755991821E-2</v>
       </c>
       <c r="I26" s="8">
-        <v>-0.1152566860974933</v>
+        <v>-1.5735104634281676</v>
       </c>
       <c r="J26" s="8">
-        <v>4.8335791804963793E-2</v>
+        <v>-1.1934464325502776</v>
       </c>
       <c r="K26" s="8">
-        <v>-0.38007554271296284</v>
+        <v>-0.85240190689112227</v>
       </c>
       <c r="L26" s="8">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="O26" s="6" t="s">
         <v>86</v>
@@ -48807,41 +48699,41 @@
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A27" s="5">
+      <c r="A27" s="7">
+        <v>0</v>
+      </c>
+      <c r="B27" s="8">
+        <v>0.67900414836397049</v>
+      </c>
+      <c r="C27" s="8">
+        <v>-1.1208996282366439</v>
+      </c>
+      <c r="D27" s="8">
+        <v>0.3790395564130048</v>
+      </c>
+      <c r="E27" s="8">
+        <v>0.77840206294000935</v>
+      </c>
+      <c r="F27" s="8">
+        <v>0.58872682173898827</v>
+      </c>
+      <c r="G27" s="8">
+        <v>0.73007771213651806</v>
+      </c>
+      <c r="H27" s="8">
+        <v>6.3862432854676188E-2</v>
+      </c>
+      <c r="I27" s="8">
+        <v>-1.867982447722611</v>
+      </c>
+      <c r="J27" s="8">
+        <v>-1.6345920430877501</v>
+      </c>
+      <c r="K27" s="8">
+        <v>-1.156702681655305</v>
+      </c>
+      <c r="L27" s="8">
         <v>1</v>
-      </c>
-      <c r="B27" s="8">
-        <v>0.40307212927502833</v>
-      </c>
-      <c r="C27" s="8">
-        <v>-0.38409278654220974</v>
-      </c>
-      <c r="D27" s="8">
-        <v>0.24286635287172137</v>
-      </c>
-      <c r="E27" s="8">
-        <v>0.36088554712190801</v>
-      </c>
-      <c r="F27" s="8">
-        <v>0.11767541403108975</v>
-      </c>
-      <c r="G27" s="8">
-        <v>0.78819312824362509</v>
-      </c>
-      <c r="H27" s="8">
-        <v>-3.4457935648817717E-2</v>
-      </c>
-      <c r="I27" s="8">
-        <v>-0.47559922109553432</v>
-      </c>
-      <c r="J27" s="8">
-        <v>-0.1390336640222814</v>
-      </c>
-      <c r="K27" s="8">
-        <v>-0.94611270969677663</v>
-      </c>
-      <c r="L27" s="8">
-        <v>5</v>
       </c>
       <c r="O27" s="6" t="s">
         <v>241</v>
@@ -48851,41 +48743,41 @@
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A28" s="6" t="s">
-        <v>86</v>
+      <c r="A28" s="7">
+        <v>1</v>
       </c>
       <c r="B28" s="8">
-        <v>0.40307212927502833</v>
+        <v>0.62314294886518273</v>
       </c>
       <c r="C28" s="8">
-        <v>-0.38409278654220974</v>
+        <v>-1.0549478242461581</v>
       </c>
       <c r="D28" s="8">
-        <v>0.24286635287172137</v>
+        <v>0.2213996632474281</v>
       </c>
       <c r="E28" s="8">
-        <v>0.36088554712190801</v>
+        <v>0.76402129048067091</v>
       </c>
       <c r="F28" s="8">
-        <v>0.11767541403108975</v>
+        <v>0.65248239848207623</v>
       </c>
       <c r="G28" s="8">
-        <v>0.78819312824362509</v>
+        <v>0.68649543169841976</v>
       </c>
       <c r="H28" s="8">
-        <v>-3.4457935648817717E-2</v>
+        <v>-0.1693866774521926</v>
       </c>
       <c r="I28" s="8">
-        <v>-0.47559922109553432</v>
+        <v>-1.669728116053067</v>
       </c>
       <c r="J28" s="8">
-        <v>-0.1390336640222814</v>
+        <v>-1.2730945595948471</v>
       </c>
       <c r="K28" s="8">
-        <v>-0.94611270969677663</v>
+        <v>-0.88404639845994981</v>
       </c>
       <c r="L28" s="8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="O28" s="6" t="s">
         <v>175</v>
@@ -48896,37 +48788,37 @@
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" s="7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B29" s="8">
-        <v>0.4265670805307275</v>
+        <v>0.63622091725460783</v>
       </c>
       <c r="C29" s="8">
-        <v>-0.56800594377510771</v>
+        <v>-1.0312736864732901</v>
       </c>
       <c r="D29" s="8">
-        <v>0.26567018161996392</v>
+        <v>0.2342815652569766</v>
       </c>
       <c r="E29" s="8">
-        <v>0.39542136922712878</v>
+        <v>0.73823531748798055</v>
       </c>
       <c r="F29" s="8">
-        <v>0.14489457713923379</v>
+        <v>0.66372060074580252</v>
       </c>
       <c r="G29" s="8">
-        <v>0.80326104224981365</v>
+        <v>0.71196298042938144</v>
       </c>
       <c r="H29" s="8">
-        <v>-0.30697220600760572</v>
+        <v>0.2942816140089406</v>
       </c>
       <c r="I29" s="8">
-        <v>-0.68315349377639945</v>
+        <v>-1.2606017679957451</v>
       </c>
       <c r="J29" s="8">
-        <v>-0.19170100301661019</v>
+        <v>-0.97183838209557361</v>
       </c>
       <c r="K29" s="8">
-        <v>-1.3208823454805869</v>
+        <v>-0.85050552639387833</v>
       </c>
       <c r="L29" s="8">
         <v>1</v>
@@ -48940,37 +48832,37 @@
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" s="7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B30" s="8">
-        <v>0.34913976236230748</v>
+        <v>0.7071204450566142</v>
       </c>
       <c r="C30" s="8">
-        <v>-0.14319329478432299</v>
+        <v>-0.92742429284550676</v>
       </c>
       <c r="D30" s="8">
-        <v>0.16876904308305879</v>
+        <v>0.52803373502828888</v>
       </c>
       <c r="E30" s="8">
-        <v>0.30962560357124702</v>
+        <v>0.76342657535949399</v>
       </c>
       <c r="F30" s="8">
-        <v>8.0092309452948429E-2</v>
+        <v>0.65083825473686563</v>
       </c>
       <c r="G30" s="8">
-        <v>0.7780452519197949</v>
+        <v>0.64822697379292327</v>
       </c>
       <c r="H30" s="8">
-        <v>0.17272212982402871</v>
+        <v>-0.33466037864722709</v>
       </c>
       <c r="I30" s="8">
-        <v>-0.2309835712801058</v>
+        <v>-1.464014056865603</v>
       </c>
       <c r="J30" s="8">
-        <v>-6.0824068280210142E-2</v>
+        <v>-1.0157773013881981</v>
       </c>
       <c r="K30" s="8">
-        <v>-0.55245686129743032</v>
+        <v>-0.44976422801388449</v>
       </c>
       <c r="L30" s="8">
         <v>1</v>
@@ -48984,37 +48876,37 @@
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B31" s="8">
-        <v>0.40270321163788242</v>
+        <v>0.64484311866941546</v>
       </c>
       <c r="C31" s="8">
-        <v>-0.36173987753704911</v>
+        <v>-0.94938369355342833</v>
       </c>
       <c r="D31" s="8">
-        <v>0.24474388669368799</v>
+        <v>0.25649082144622781</v>
       </c>
       <c r="E31" s="8">
-        <v>0.35186930212477052</v>
+        <v>0.78866292355203438</v>
       </c>
       <c r="F31" s="8">
-        <v>0.1252465789378607</v>
+        <v>0.65642544427209859</v>
       </c>
       <c r="G31" s="8">
-        <v>0.78029832059154924</v>
+        <v>0.70055975105268931</v>
       </c>
       <c r="H31" s="8">
-        <v>-0.15506311711034779</v>
+        <v>-0.1229145795441562</v>
       </c>
       <c r="I31" s="8">
-        <v>-0.34010410849117578</v>
+        <v>-1.605225928503812</v>
       </c>
       <c r="J31" s="8">
-        <v>-8.9886049829636328E-2</v>
+        <v>-1.07192987658502</v>
       </c>
       <c r="K31" s="8">
-        <v>-0.77157729202631997</v>
+        <v>-0.92099069993259364</v>
       </c>
       <c r="L31" s="8">
         <v>1</v>
@@ -49027,41 +48919,41 @@
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A32" s="7">
+      <c r="A32" s="5">
         <v>3</v>
       </c>
       <c r="B32" s="8">
-        <v>0.41227629571046143</v>
+        <v>0.4741805704078903</v>
       </c>
       <c r="C32" s="8">
-        <v>-0.35117530143303433</v>
+        <v>-0.17434896788740781</v>
       </c>
       <c r="D32" s="8">
-        <v>0.25532204503223749</v>
+        <v>0.11378058804706315</v>
       </c>
       <c r="E32" s="8">
-        <v>0.35980052369876431</v>
+        <v>0.61562676263409788</v>
       </c>
       <c r="F32" s="8">
-        <v>0.1168874035781555</v>
+        <v>0.59872345506574054</v>
       </c>
       <c r="G32" s="8">
-        <v>0.79105514782979947</v>
+        <v>0.42791169102775672</v>
       </c>
       <c r="H32" s="8">
-        <v>7.1535294243375125E-2</v>
+        <v>-0.15357090852365513</v>
       </c>
       <c r="I32" s="8">
-        <v>-0.45395816669139721</v>
+        <v>-0.20130165107118447</v>
       </c>
       <c r="J32" s="8">
-        <v>-0.15758815650815319</v>
+        <v>-0.25086429603928662</v>
       </c>
       <c r="K32" s="8">
-        <v>-0.79379475304162295</v>
+        <v>-6.9471857962544709E-2</v>
       </c>
       <c r="L32" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O32" s="6" t="s">
         <v>141</v>
@@ -49071,41 +48963,41 @@
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A33" s="7">
-        <v>4</v>
+      <c r="A33" s="5">
+        <v>5</v>
       </c>
       <c r="B33" s="8">
-        <v>0.42467429613376301</v>
+        <v>0.3000109637759224</v>
       </c>
       <c r="C33" s="8">
-        <v>-0.49634951518153458</v>
+        <v>-9.4938328357782625E-2</v>
       </c>
       <c r="D33" s="8">
-        <v>0.27982660792965869</v>
+        <v>-1.4759654499295371E-2</v>
       </c>
       <c r="E33" s="8">
-        <v>0.38771093698762937</v>
+        <v>0.42900186041466259</v>
       </c>
       <c r="F33" s="8">
-        <v>0.12125620104725029</v>
+        <v>0.48723375792125767</v>
       </c>
       <c r="G33" s="8">
-        <v>0.78830587862716817</v>
+        <v>0.23329104366752945</v>
       </c>
       <c r="H33" s="8">
-        <v>4.5488220806461088E-2</v>
+        <v>-6.4232437311530236E-2</v>
       </c>
       <c r="I33" s="8">
-        <v>-0.66979676523859322</v>
+        <v>-8.4360392897282879E-2</v>
       </c>
       <c r="J33" s="8">
-        <v>-0.19516904247679709</v>
+        <v>-0.14400159382853714</v>
       </c>
       <c r="K33" s="8">
-        <v>-1.2918522966379229</v>
+        <v>-0.1103670511867975</v>
       </c>
       <c r="L33" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O33" s="6" t="s">
         <v>158</v>
@@ -49115,1415 +49007,47 @@
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A34" s="5">
-        <v>3</v>
+      <c r="A34" s="4" t="s">
+        <v>280</v>
       </c>
       <c r="B34" s="8">
-        <v>0.44214423893222754</v>
+        <v>0.40845973549716619</v>
       </c>
       <c r="C34" s="8">
-        <v>5.9381069547292865E-2</v>
+        <v>-0.22851485149413822</v>
       </c>
       <c r="D34" s="8">
-        <v>0.10824553380471022</v>
+        <v>0.13961569356052095</v>
       </c>
       <c r="E34" s="8">
-        <v>0.47664456889684359</v>
+        <v>0.4780866463891581</v>
       </c>
       <c r="F34" s="8">
-        <v>0.38540290740041361</v>
+        <v>0.41283913785817766</v>
       </c>
       <c r="G34" s="8">
-        <v>0.66212392028841749</v>
+        <v>0.49667331417674704</v>
       </c>
       <c r="H34" s="8">
-        <v>-0.11002622203250137</v>
+        <v>-6.458582977373914E-2</v>
       </c>
       <c r="I34" s="8">
-        <v>0.13499579743245385</v>
+        <v>-0.30841822468824392</v>
       </c>
       <c r="J34" s="8">
-        <v>0.20226114065201303</v>
+        <v>-0.21568113252070364</v>
       </c>
       <c r="K34" s="8">
-        <v>-2.0336451665511103E-2</v>
+        <v>-0.28072662168981544</v>
       </c>
       <c r="L34" s="8">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="O34" s="4" t="s">
         <v>280</v>
       </c>
       <c r="P34">
         <v>0.32446283165088879</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A35" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="B35" s="8">
-        <v>0.44214423893222754</v>
-      </c>
-      <c r="C35" s="8">
-        <v>5.9381069547292865E-2</v>
-      </c>
-      <c r="D35" s="8">
-        <v>0.10824553380471022</v>
-      </c>
-      <c r="E35" s="8">
-        <v>0.47664456889684359</v>
-      </c>
-      <c r="F35" s="8">
-        <v>0.38540290740041361</v>
-      </c>
-      <c r="G35" s="8">
-        <v>0.66212392028841749</v>
-      </c>
-      <c r="H35" s="8">
-        <v>-0.11002622203250137</v>
-      </c>
-      <c r="I35" s="8">
-        <v>0.13499579743245385</v>
-      </c>
-      <c r="J35" s="8">
-        <v>0.20226114065201303</v>
-      </c>
-      <c r="K35" s="8">
-        <v>-2.0336451665511103E-2</v>
-      </c>
-      <c r="L35" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A36" s="7">
-        <v>0</v>
-      </c>
-      <c r="B36" s="8">
-        <v>0.45395891905647789</v>
-      </c>
-      <c r="C36" s="8">
-        <v>0.124929981065744</v>
-      </c>
-      <c r="D36" s="8">
-        <v>-1.809764503878775E-2</v>
-      </c>
-      <c r="E36" s="8">
-        <v>0.56801500224344492</v>
-      </c>
-      <c r="F36" s="8">
-        <v>0.40332804000037242</v>
-      </c>
-      <c r="G36" s="8">
-        <v>0.67477633144171989</v>
-      </c>
-      <c r="H36" s="8">
-        <v>-7.9495977739627577E-2</v>
-      </c>
-      <c r="I36" s="8">
-        <v>0.1991450126619172</v>
-      </c>
-      <c r="J36" s="8">
-        <v>0.29665984604229018</v>
-      </c>
-      <c r="K36" s="8">
-        <v>-6.0228607546063628E-2</v>
-      </c>
-      <c r="L36" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A37" s="7">
-        <v>1</v>
-      </c>
-      <c r="B37" s="8">
-        <v>0.42544640928094579</v>
-      </c>
-      <c r="C37" s="8">
-        <v>-7.2588215486826507E-2</v>
-      </c>
-      <c r="D37" s="8">
-        <v>0.14399313074154291</v>
-      </c>
-      <c r="E37" s="8">
-        <v>0.40109522160835609</v>
-      </c>
-      <c r="F37" s="8">
-        <v>0.33335781556025629</v>
-      </c>
-      <c r="G37" s="8">
-        <v>0.67519230228000304</v>
-      </c>
-      <c r="H37" s="8">
-        <v>-0.172800687123146</v>
-      </c>
-      <c r="I37" s="8">
-        <v>-5.666822167024077E-2</v>
-      </c>
-      <c r="J37" s="8">
-        <v>-1.7230247769852051E-2</v>
-      </c>
-      <c r="K37" s="8">
-        <v>-1.9180866768028441E-2</v>
-      </c>
-      <c r="L37" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A38" s="7">
-        <v>2</v>
-      </c>
-      <c r="B38" s="8">
-        <v>0.5135118984289756</v>
-      </c>
-      <c r="C38" s="8">
-        <v>0.1115264238927912</v>
-      </c>
-      <c r="D38" s="8">
-        <v>0.21578363024716929</v>
-      </c>
-      <c r="E38" s="8">
-        <v>0.52980454279926414</v>
-      </c>
-      <c r="F38" s="8">
-        <v>0.47042277488149531</v>
-      </c>
-      <c r="G38" s="8">
-        <v>0.6660622753944565</v>
-      </c>
-      <c r="H38" s="8">
-        <v>-0.1202751126222841</v>
-      </c>
-      <c r="I38" s="8">
-        <v>0.2003477252240996</v>
-      </c>
-      <c r="J38" s="8">
-        <v>0.31113842653827117</v>
-      </c>
-      <c r="K38" s="8">
-        <v>3.6290827666484171E-3</v>
-      </c>
-      <c r="L38" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A39" s="7">
-        <v>3</v>
-      </c>
-      <c r="B39" s="8">
-        <v>0.39560503601946201</v>
-      </c>
-      <c r="C39" s="8">
-        <v>0.1107517653212195</v>
-      </c>
-      <c r="D39" s="8">
-        <v>5.4009397928678538E-2</v>
-      </c>
-      <c r="E39" s="8">
-        <v>0.44515599889020008</v>
-      </c>
-      <c r="F39" s="8">
-        <v>0.33278512794233978</v>
-      </c>
-      <c r="G39" s="8">
-        <v>0.63813339106651257</v>
-      </c>
-      <c r="H39" s="8">
-        <v>-4.609684054032881E-2</v>
-      </c>
-      <c r="I39" s="8">
-        <v>0.14198905306334639</v>
-      </c>
-      <c r="J39" s="8">
-        <v>0.22582309851941859</v>
-      </c>
-      <c r="K39" s="8">
-        <v>-5.2530100901335468E-2</v>
-      </c>
-      <c r="L39" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A40" s="7">
-        <v>4</v>
-      </c>
-      <c r="B40" s="8">
-        <v>0.42219893187527657</v>
-      </c>
-      <c r="C40" s="8">
-        <v>2.2285392943536101E-2</v>
-      </c>
-      <c r="D40" s="8">
-        <v>0.1455391551449482</v>
-      </c>
-      <c r="E40" s="8">
-        <v>0.43915207894295272</v>
-      </c>
-      <c r="F40" s="8">
-        <v>0.38712077861760402</v>
-      </c>
-      <c r="G40" s="8">
-        <v>0.65645530125939544</v>
-      </c>
-      <c r="H40" s="8">
-        <v>-0.13146249213712041</v>
-      </c>
-      <c r="I40" s="8">
-        <v>0.19016541788314681</v>
-      </c>
-      <c r="J40" s="8">
-        <v>0.19491457992993741</v>
-      </c>
-      <c r="K40" s="8">
-        <v>2.6628234121223619E-2</v>
-      </c>
-      <c r="L40" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A41" s="5">
-        <v>5</v>
-      </c>
-      <c r="B41" s="8">
-        <v>0.37825163831724673</v>
-      </c>
-      <c r="C41" s="8">
-        <v>-1.1440306533764349E-2</v>
-      </c>
-      <c r="D41" s="8">
-        <v>0.11364682961159425</v>
-      </c>
-      <c r="E41" s="8">
-        <v>0.3907120300698248</v>
-      </c>
-      <c r="F41" s="8">
-        <v>0.26533640745113807</v>
-      </c>
-      <c r="G41" s="8">
-        <v>0.60895783733343389</v>
-      </c>
-      <c r="H41" s="8">
-        <v>-1.8615006906109999E-2</v>
-      </c>
-      <c r="I41" s="8">
-        <v>-5.1666346293995965E-3</v>
-      </c>
-      <c r="J41" s="8">
-        <v>8.1779898785159691E-2</v>
-      </c>
-      <c r="K41" s="8">
-        <v>-0.17377746677660094</v>
-      </c>
-      <c r="L41" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A42" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="B42" s="8">
-        <v>0.37825163831724673</v>
-      </c>
-      <c r="C42" s="8">
-        <v>-1.1440306533764349E-2</v>
-      </c>
-      <c r="D42" s="8">
-        <v>0.11364682961159425</v>
-      </c>
-      <c r="E42" s="8">
-        <v>0.3907120300698248</v>
-      </c>
-      <c r="F42" s="8">
-        <v>0.26533640745113807</v>
-      </c>
-      <c r="G42" s="8">
-        <v>0.60895783733343389</v>
-      </c>
-      <c r="H42" s="8">
-        <v>-1.8615006906109999E-2</v>
-      </c>
-      <c r="I42" s="8">
-        <v>-5.1666346293995965E-3</v>
-      </c>
-      <c r="J42" s="8">
-        <v>8.1779898785159691E-2</v>
-      </c>
-      <c r="K42" s="8">
-        <v>-0.17377746677660094</v>
-      </c>
-      <c r="L42" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A43" s="7">
-        <v>0</v>
-      </c>
-      <c r="B43" s="8">
-        <v>0.37347365362292828</v>
-      </c>
-      <c r="C43" s="8">
-        <v>4.5593102251826501E-2</v>
-      </c>
-      <c r="D43" s="8">
-        <v>8.9079143663578497E-2</v>
-      </c>
-      <c r="E43" s="8">
-        <v>0.33604024964342338</v>
-      </c>
-      <c r="F43" s="8">
-        <v>0.20574857695664051</v>
-      </c>
-      <c r="G43" s="8">
-        <v>0.66300720842047789</v>
-      </c>
-      <c r="H43" s="8">
-        <v>-7.9528360879142612E-2</v>
-      </c>
-      <c r="I43" s="8">
-        <v>0.11947831492600169</v>
-      </c>
-      <c r="J43" s="8">
-        <v>0.1160033818969346</v>
-      </c>
-      <c r="K43" s="8">
-        <v>-0.1210838025025021</v>
-      </c>
-      <c r="L43" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A44" s="7">
-        <v>1</v>
-      </c>
-      <c r="B44" s="8">
-        <v>0.32419610479266592</v>
-      </c>
-      <c r="C44" s="8">
-        <v>-5.6605278111632101E-2</v>
-      </c>
-      <c r="D44" s="8">
-        <v>0.1764680445576354</v>
-      </c>
-      <c r="E44" s="8">
-        <v>0.27742806059839942</v>
-      </c>
-      <c r="F44" s="8">
-        <v>0.1187028298739924</v>
-      </c>
-      <c r="G44" s="8">
-        <v>0.5555610896311669</v>
-      </c>
-      <c r="H44" s="8">
-        <v>2.9126536491069781E-3</v>
-      </c>
-      <c r="I44" s="8">
-        <v>-3.7005753887184627E-2</v>
-      </c>
-      <c r="J44" s="8">
-        <v>2.4202653038465249E-2</v>
-      </c>
-      <c r="K44" s="8">
-        <v>-0.25810162613625542</v>
-      </c>
-      <c r="L44" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A45" s="7">
-        <v>2</v>
-      </c>
-      <c r="B45" s="8">
-        <v>0.35910691736394479</v>
-      </c>
-      <c r="C45" s="8">
-        <v>-6.4947118630907213E-2</v>
-      </c>
-      <c r="D45" s="8">
-        <v>0.1225929397635995</v>
-      </c>
-      <c r="E45" s="8">
-        <v>0.41160711763952668</v>
-      </c>
-      <c r="F45" s="8">
-        <v>0.25056136125221901</v>
-      </c>
-      <c r="G45" s="8">
-        <v>0.64113163383465277</v>
-      </c>
-      <c r="H45" s="8">
-        <v>-3.5184485113790347E-2</v>
-      </c>
-      <c r="I45" s="8">
-        <v>-3.4124824750739302E-2</v>
-      </c>
-      <c r="J45" s="8">
-        <v>1.0620097819174281E-2</v>
-      </c>
-      <c r="K45" s="8">
-        <v>-0.17357964195241979</v>
-      </c>
-      <c r="L45" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A46" s="7">
-        <v>3</v>
-      </c>
-      <c r="B46" s="8">
-        <v>0.3778227144642663</v>
-      </c>
-      <c r="C46" s="8">
-        <v>-5.0844541917639818E-2</v>
-      </c>
-      <c r="D46" s="8">
-        <v>0.13177575770574179</v>
-      </c>
-      <c r="E46" s="8">
-        <v>0.36868605296648288</v>
-      </c>
-      <c r="F46" s="8">
-        <v>0.24281434646440539</v>
-      </c>
-      <c r="G46" s="8">
-        <v>0.61050651304286818</v>
-      </c>
-      <c r="H46" s="8">
-        <v>3.9635246664473052E-2</v>
-      </c>
-      <c r="I46" s="8">
-        <v>-0.14708900532620109</v>
-      </c>
-      <c r="J46" s="8">
-        <v>1.9168896179289069E-4</v>
-      </c>
-      <c r="K46" s="8">
-        <v>-0.16915474515971279</v>
-      </c>
-      <c r="L46" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A47" s="7">
-        <v>4</v>
-      </c>
-      <c r="B47" s="8">
-        <v>0.45665880134242848</v>
-      </c>
-      <c r="C47" s="8">
-        <v>6.9602303739530885E-2</v>
-      </c>
-      <c r="D47" s="8">
-        <v>4.8318262367415987E-2</v>
-      </c>
-      <c r="E47" s="8">
-        <v>0.55979866950129176</v>
-      </c>
-      <c r="F47" s="8">
-        <v>0.50885492270843313</v>
-      </c>
-      <c r="G47" s="8">
-        <v>0.57458274173800405</v>
-      </c>
-      <c r="H47" s="8">
-        <v>-2.0910088851197051E-2</v>
-      </c>
-      <c r="I47" s="8">
-        <v>7.2908095891125346E-2</v>
-      </c>
-      <c r="J47" s="8">
-        <v>0.25788167220943142</v>
-      </c>
-      <c r="K47" s="8">
-        <v>-0.14696751813211459</v>
-      </c>
-      <c r="L47" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A48" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B48" s="8">
-        <v>0.47741928327525696</v>
-      </c>
-      <c r="C48" s="8">
-        <v>-0.42869104043873196</v>
-      </c>
-      <c r="D48" s="8">
-        <v>0.14095666727538436</v>
-      </c>
-      <c r="E48" s="8">
-        <v>0.60372608567093289</v>
-      </c>
-      <c r="F48" s="8">
-        <v>0.57613197232738822</v>
-      </c>
-      <c r="G48" s="8">
-        <v>0.45222243483909075</v>
-      </c>
-      <c r="H48" s="8">
-        <v>-9.0522287863725737E-2</v>
-      </c>
-      <c r="I48" s="8">
-        <v>-0.61972416913221184</v>
-      </c>
-      <c r="J48" s="8">
-        <v>-0.52943744080603383</v>
-      </c>
-      <c r="K48" s="8">
-        <v>-0.34408027201348812</v>
-      </c>
-      <c r="L48" s="8">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A49" s="5">
-        <v>1</v>
-      </c>
-      <c r="B49" s="8">
-        <v>0.65806631564195817</v>
-      </c>
-      <c r="C49" s="8">
-        <v>-1.0167858250710053</v>
-      </c>
-      <c r="D49" s="8">
-        <v>0.32384906827838522</v>
-      </c>
-      <c r="E49" s="8">
-        <v>0.76654963396403786</v>
-      </c>
-      <c r="F49" s="8">
-        <v>0.64243870399516623</v>
-      </c>
-      <c r="G49" s="8">
-        <v>0.69546456982198634</v>
-      </c>
-      <c r="H49" s="8">
-        <v>-5.3763517755991821E-2</v>
-      </c>
-      <c r="I49" s="8">
-        <v>-1.5735104634281676</v>
-      </c>
-      <c r="J49" s="8">
-        <v>-1.1934464325502776</v>
-      </c>
-      <c r="K49" s="8">
-        <v>-0.85240190689112227</v>
-      </c>
-      <c r="L49" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A50" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="B50" s="8">
-        <v>0.65806631564195817</v>
-      </c>
-      <c r="C50" s="8">
-        <v>-1.0167858250710053</v>
-      </c>
-      <c r="D50" s="8">
-        <v>0.32384906827838522</v>
-      </c>
-      <c r="E50" s="8">
-        <v>0.76654963396403786</v>
-      </c>
-      <c r="F50" s="8">
-        <v>0.64243870399516623</v>
-      </c>
-      <c r="G50" s="8">
-        <v>0.69546456982198634</v>
-      </c>
-      <c r="H50" s="8">
-        <v>-5.3763517755991821E-2</v>
-      </c>
-      <c r="I50" s="8">
-        <v>-1.5735104634281676</v>
-      </c>
-      <c r="J50" s="8">
-        <v>-1.1934464325502776</v>
-      </c>
-      <c r="K50" s="8">
-        <v>-0.85240190689112227</v>
-      </c>
-      <c r="L50" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A51" s="7">
-        <v>0</v>
-      </c>
-      <c r="B51" s="8">
-        <v>0.67900414836397049</v>
-      </c>
-      <c r="C51" s="8">
-        <v>-1.1208996282366439</v>
-      </c>
-      <c r="D51" s="8">
-        <v>0.3790395564130048</v>
-      </c>
-      <c r="E51" s="8">
-        <v>0.77840206294000935</v>
-      </c>
-      <c r="F51" s="8">
-        <v>0.58872682173898827</v>
-      </c>
-      <c r="G51" s="8">
-        <v>0.73007771213651806</v>
-      </c>
-      <c r="H51" s="8">
-        <v>6.3862432854676188E-2</v>
-      </c>
-      <c r="I51" s="8">
-        <v>-1.867982447722611</v>
-      </c>
-      <c r="J51" s="8">
-        <v>-1.6345920430877501</v>
-      </c>
-      <c r="K51" s="8">
-        <v>-1.156702681655305</v>
-      </c>
-      <c r="L51" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A52" s="7">
-        <v>1</v>
-      </c>
-      <c r="B52" s="8">
-        <v>0.62314294886518273</v>
-      </c>
-      <c r="C52" s="8">
-        <v>-1.0549478242461581</v>
-      </c>
-      <c r="D52" s="8">
-        <v>0.2213996632474281</v>
-      </c>
-      <c r="E52" s="8">
-        <v>0.76402129048067091</v>
-      </c>
-      <c r="F52" s="8">
-        <v>0.65248239848207623</v>
-      </c>
-      <c r="G52" s="8">
-        <v>0.68649543169841976</v>
-      </c>
-      <c r="H52" s="8">
-        <v>-0.1693866774521926</v>
-      </c>
-      <c r="I52" s="8">
-        <v>-1.669728116053067</v>
-      </c>
-      <c r="J52" s="8">
-        <v>-1.2730945595948471</v>
-      </c>
-      <c r="K52" s="8">
-        <v>-0.88404639845994981</v>
-      </c>
-      <c r="L52" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A53" s="7">
-        <v>2</v>
-      </c>
-      <c r="B53" s="8">
-        <v>0.63622091725460783</v>
-      </c>
-      <c r="C53" s="8">
-        <v>-1.0312736864732901</v>
-      </c>
-      <c r="D53" s="8">
-        <v>0.2342815652569766</v>
-      </c>
-      <c r="E53" s="8">
-        <v>0.73823531748798055</v>
-      </c>
-      <c r="F53" s="8">
-        <v>0.66372060074580252</v>
-      </c>
-      <c r="G53" s="8">
-        <v>0.71196298042938144</v>
-      </c>
-      <c r="H53" s="8">
-        <v>0.2942816140089406</v>
-      </c>
-      <c r="I53" s="8">
-        <v>-1.2606017679957451</v>
-      </c>
-      <c r="J53" s="8">
-        <v>-0.97183838209557361</v>
-      </c>
-      <c r="K53" s="8">
-        <v>-0.85050552639387833</v>
-      </c>
-      <c r="L53" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A54" s="7">
-        <v>3</v>
-      </c>
-      <c r="B54" s="8">
-        <v>0.7071204450566142</v>
-      </c>
-      <c r="C54" s="8">
-        <v>-0.92742429284550676</v>
-      </c>
-      <c r="D54" s="8">
-        <v>0.52803373502828888</v>
-      </c>
-      <c r="E54" s="8">
-        <v>0.76342657535949399</v>
-      </c>
-      <c r="F54" s="8">
-        <v>0.65083825473686563</v>
-      </c>
-      <c r="G54" s="8">
-        <v>0.64822697379292327</v>
-      </c>
-      <c r="H54" s="8">
-        <v>-0.33466037864722709</v>
-      </c>
-      <c r="I54" s="8">
-        <v>-1.464014056865603</v>
-      </c>
-      <c r="J54" s="8">
-        <v>-1.0157773013881981</v>
-      </c>
-      <c r="K54" s="8">
-        <v>-0.44976422801388449</v>
-      </c>
-      <c r="L54" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A55" s="7">
-        <v>4</v>
-      </c>
-      <c r="B55" s="8">
-        <v>0.64484311866941546</v>
-      </c>
-      <c r="C55" s="8">
-        <v>-0.94938369355342833</v>
-      </c>
-      <c r="D55" s="8">
-        <v>0.25649082144622781</v>
-      </c>
-      <c r="E55" s="8">
-        <v>0.78866292355203438</v>
-      </c>
-      <c r="F55" s="8">
-        <v>0.65642544427209859</v>
-      </c>
-      <c r="G55" s="8">
-        <v>0.70055975105268931</v>
-      </c>
-      <c r="H55" s="8">
-        <v>-0.1229145795441562</v>
-      </c>
-      <c r="I55" s="8">
-        <v>-1.605225928503812</v>
-      </c>
-      <c r="J55" s="8">
-        <v>-1.07192987658502</v>
-      </c>
-      <c r="K55" s="8">
-        <v>-0.92099069993259364</v>
-      </c>
-      <c r="L55" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A56" s="5">
-        <v>3</v>
-      </c>
-      <c r="B56" s="8">
-        <v>0.4741805704078903</v>
-      </c>
-      <c r="C56" s="8">
-        <v>-0.17434896788740781</v>
-      </c>
-      <c r="D56" s="8">
-        <v>0.11378058804706315</v>
-      </c>
-      <c r="E56" s="8">
-        <v>0.61562676263409788</v>
-      </c>
-      <c r="F56" s="8">
-        <v>0.59872345506574065</v>
-      </c>
-      <c r="G56" s="8">
-        <v>0.42791169102775672</v>
-      </c>
-      <c r="H56" s="8">
-        <v>-0.15357090852365513</v>
-      </c>
-      <c r="I56" s="8">
-        <v>-0.20130165107118447</v>
-      </c>
-      <c r="J56" s="8">
-        <v>-0.25086429603928662</v>
-      </c>
-      <c r="K56" s="8">
-        <v>-6.9471857962544709E-2</v>
-      </c>
-      <c r="L56" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A57" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="B57" s="8">
-        <v>0.4741805704078903</v>
-      </c>
-      <c r="C57" s="8">
-        <v>-0.17434896788740781</v>
-      </c>
-      <c r="D57" s="8">
-        <v>0.11378058804706315</v>
-      </c>
-      <c r="E57" s="8">
-        <v>0.61562676263409788</v>
-      </c>
-      <c r="F57" s="8">
-        <v>0.59872345506574065</v>
-      </c>
-      <c r="G57" s="8">
-        <v>0.42791169102775672</v>
-      </c>
-      <c r="H57" s="8">
-        <v>-0.15357090852365513</v>
-      </c>
-      <c r="I57" s="8">
-        <v>-0.20130165107118447</v>
-      </c>
-      <c r="J57" s="8">
-        <v>-0.25086429603928662</v>
-      </c>
-      <c r="K57" s="8">
-        <v>-6.9471857962544709E-2</v>
-      </c>
-      <c r="L57" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A58" s="7">
-        <v>0</v>
-      </c>
-      <c r="B58" s="8">
-        <v>0.45665634681662148</v>
-      </c>
-      <c r="C58" s="8">
-        <v>-0.19173383937670421</v>
-      </c>
-      <c r="D58" s="8">
-        <v>0.16981386518239569</v>
-      </c>
-      <c r="E58" s="8">
-        <v>0.62912880250921965</v>
-      </c>
-      <c r="F58" s="8">
-        <v>0.58011284957378828</v>
-      </c>
-      <c r="G58" s="8">
-        <v>0.34964288359858209</v>
-      </c>
-      <c r="H58" s="8">
-        <v>-0.21790284359136769</v>
-      </c>
-      <c r="I58" s="8">
-        <v>-0.1086852264636473</v>
-      </c>
-      <c r="J58" s="8">
-        <v>-0.2048895966725619</v>
-      </c>
-      <c r="K58" s="8">
-        <v>-0.1218008594717432</v>
-      </c>
-      <c r="L58" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A59" s="7">
-        <v>1</v>
-      </c>
-      <c r="B59" s="8">
-        <v>0.42674085143399548</v>
-      </c>
-      <c r="C59" s="8">
-        <v>-3.0434908247640089E-2</v>
-      </c>
-      <c r="D59" s="8">
-        <v>6.0908005911953667E-2</v>
-      </c>
-      <c r="E59" s="8">
-        <v>0.5379463968387409</v>
-      </c>
-      <c r="F59" s="8">
-        <v>0.55080342103604363</v>
-      </c>
-      <c r="G59" s="8">
-        <v>0.44377815079484711</v>
-      </c>
-      <c r="H59" s="8">
-        <v>-0.15729280305632901</v>
-      </c>
-      <c r="I59" s="8">
-        <v>0.1006210399107894</v>
-      </c>
-      <c r="J59" s="8">
-        <v>-4.8276196955280293E-2</v>
-      </c>
-      <c r="K59" s="8">
-        <v>-4.0189122836042479E-2</v>
-      </c>
-      <c r="L59" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A60" s="7">
-        <v>2</v>
-      </c>
-      <c r="B60" s="8">
-        <v>0.51328633309388549</v>
-      </c>
-      <c r="C60" s="8">
-        <v>-0.33485559165210449</v>
-      </c>
-      <c r="D60" s="8">
-        <v>0.1178284790306698</v>
-      </c>
-      <c r="E60" s="8">
-        <v>0.66531496383135713</v>
-      </c>
-      <c r="F60" s="8">
-        <v>0.66673678843345496</v>
-      </c>
-      <c r="G60" s="8">
-        <v>0.47190941571804967</v>
-      </c>
-      <c r="H60" s="8">
-        <v>-0.14682148890394139</v>
-      </c>
-      <c r="I60" s="8">
-        <v>-0.64880519612023901</v>
-      </c>
-      <c r="J60" s="8">
-        <v>-0.62265643721164987</v>
-      </c>
-      <c r="K60" s="8">
-        <v>-5.269620368280048E-3</v>
-      </c>
-      <c r="L60" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A61" s="7">
-        <v>3</v>
-      </c>
-      <c r="B61" s="8">
-        <v>0.48946305705201981</v>
-      </c>
-      <c r="C61" s="8">
-        <v>-0.25886770301925971</v>
-      </c>
-      <c r="D61" s="8">
-        <v>0.1024414854510699</v>
-      </c>
-      <c r="E61" s="8">
-        <v>0.66599846087709236</v>
-      </c>
-      <c r="F61" s="8">
-        <v>0.62312304189058909</v>
-      </c>
-      <c r="G61" s="8">
-        <v>0.45589465626384051</v>
-      </c>
-      <c r="H61" s="8">
-        <v>-7.9208039145687748E-2</v>
-      </c>
-      <c r="I61" s="8">
-        <v>-0.4260692706358904</v>
-      </c>
-      <c r="J61" s="8">
-        <v>-0.41590606095081611</v>
-      </c>
-      <c r="K61" s="8">
-        <v>-0.11736805213123259</v>
-      </c>
-      <c r="L61" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A62" s="7">
-        <v>4</v>
-      </c>
-      <c r="B62" s="8">
-        <v>0.48475626364292901</v>
-      </c>
-      <c r="C62" s="8">
-        <v>-5.585279714133054E-2</v>
-      </c>
-      <c r="D62" s="8">
-        <v>0.1179111046592267</v>
-      </c>
-      <c r="E62" s="8">
-        <v>0.57974518911407935</v>
-      </c>
-      <c r="F62" s="8">
-        <v>0.57284117439482718</v>
-      </c>
-      <c r="G62" s="8">
-        <v>0.41833334876346417</v>
-      </c>
-      <c r="H62" s="8">
-        <v>-0.16662936792094979</v>
-      </c>
-      <c r="I62" s="8">
-        <v>7.6430397953064944E-2</v>
-      </c>
-      <c r="J62" s="8">
-        <v>3.7406811593875038E-2</v>
-      </c>
-      <c r="K62" s="8">
-        <v>-6.2731635005425224E-2</v>
-      </c>
-      <c r="L62" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A63" s="5">
-        <v>5</v>
-      </c>
-      <c r="B63" s="8">
-        <v>0.3000109637759224</v>
-      </c>
-      <c r="C63" s="8">
-        <v>-9.4938328357782625E-2</v>
-      </c>
-      <c r="D63" s="8">
-        <v>-1.4759654499295371E-2</v>
-      </c>
-      <c r="E63" s="8">
-        <v>0.42900186041466259</v>
-      </c>
-      <c r="F63" s="8">
-        <v>0.48723375792125767</v>
-      </c>
-      <c r="G63" s="8">
-        <v>0.23329104366752945</v>
-      </c>
-      <c r="H63" s="8">
-        <v>-6.4232437311530236E-2</v>
-      </c>
-      <c r="I63" s="8">
-        <v>-8.4360392897282879E-2</v>
-      </c>
-      <c r="J63" s="8">
-        <v>-0.14400159382853714</v>
-      </c>
-      <c r="K63" s="8">
-        <v>-0.1103670511867975</v>
-      </c>
-      <c r="L63" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A64" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="B64" s="8">
-        <v>0.3000109637759224</v>
-      </c>
-      <c r="C64" s="8">
-        <v>-9.4938328357782625E-2</v>
-      </c>
-      <c r="D64" s="8">
-        <v>-1.4759654499295371E-2</v>
-      </c>
-      <c r="E64" s="8">
-        <v>0.42900186041466259</v>
-      </c>
-      <c r="F64" s="8">
-        <v>0.48723375792125767</v>
-      </c>
-      <c r="G64" s="8">
-        <v>0.23329104366752945</v>
-      </c>
-      <c r="H64" s="8">
-        <v>-6.4232437311530236E-2</v>
-      </c>
-      <c r="I64" s="8">
-        <v>-8.4360392897282879E-2</v>
-      </c>
-      <c r="J64" s="8">
-        <v>-0.14400159382853714</v>
-      </c>
-      <c r="K64" s="8">
-        <v>-0.1103670511867975</v>
-      </c>
-      <c r="L64" s="8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A65" s="7">
-        <v>0</v>
-      </c>
-      <c r="B65" s="8">
-        <v>0.29472064533716358</v>
-      </c>
-      <c r="C65" s="8">
-        <v>-6.0568916326290252E-2</v>
-      </c>
-      <c r="D65" s="8">
-        <v>-5.1922740934040368E-2</v>
-      </c>
-      <c r="E65" s="8">
-        <v>0.38468868386302368</v>
-      </c>
-      <c r="F65" s="8">
-        <v>0.49511570382507192</v>
-      </c>
-      <c r="G65" s="8">
-        <v>0.1831658397364139</v>
-      </c>
-      <c r="H65" s="8">
-        <v>-0.1223331478419858</v>
-      </c>
-      <c r="I65" s="8">
-        <v>-9.9681756610288108E-3</v>
-      </c>
-      <c r="J65" s="8">
-        <v>-2.3305811210891921E-2</v>
-      </c>
-      <c r="K65" s="8">
-        <v>-0.12268302898125109</v>
-      </c>
-      <c r="L65" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A66" s="7">
-        <v>1</v>
-      </c>
-      <c r="B66" s="8">
-        <v>0.29636521393145587</v>
-      </c>
-      <c r="C66" s="8">
-        <v>-0.13024197825470629</v>
-      </c>
-      <c r="D66" s="8">
-        <v>6.6856976591836204E-2</v>
-      </c>
-      <c r="E66" s="8">
-        <v>0.45767407459611842</v>
-      </c>
-      <c r="F66" s="8">
-        <v>0.57340348296019483</v>
-      </c>
-      <c r="G66" s="8">
-        <v>0.17998985060900741</v>
-      </c>
-      <c r="H66" s="8">
-        <v>4.4647554846952153E-2</v>
-      </c>
-      <c r="I66" s="8">
-        <v>-0.14951146491676839</v>
-      </c>
-      <c r="J66" s="8">
-        <v>-0.20191687223327581</v>
-      </c>
-      <c r="K66" s="8">
-        <v>-7.2074112020869219E-2</v>
-      </c>
-      <c r="L66" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A67" s="7">
-        <v>2</v>
-      </c>
-      <c r="B67" s="8">
-        <v>0.32383973594845439</v>
-      </c>
-      <c r="C67" s="8">
-        <v>-4.2251562209794653E-2</v>
-      </c>
-      <c r="D67" s="8">
-        <v>1.968322704007153E-2</v>
-      </c>
-      <c r="E67" s="8">
-        <v>0.46963080380879879</v>
-      </c>
-      <c r="F67" s="8">
-        <v>0.44883202914765241</v>
-      </c>
-      <c r="G67" s="8">
-        <v>0.32262650102711438</v>
-      </c>
-      <c r="H67" s="8">
-        <v>-8.5295567127336547E-2</v>
-      </c>
-      <c r="I67" s="8">
-        <v>-6.2874332835315183E-2</v>
-      </c>
-      <c r="J67" s="8">
-        <v>-8.8211705491311188E-2</v>
-      </c>
-      <c r="K67" s="8">
-        <v>-5.4208758561032473E-2</v>
-      </c>
-      <c r="L67" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A68" s="7">
-        <v>3</v>
-      </c>
-      <c r="B68" s="8">
-        <v>0.2548188836247523</v>
-      </c>
-      <c r="C68" s="8">
-        <v>-3.9599406230942047E-2</v>
-      </c>
-      <c r="D68" s="8">
-        <v>-3.8919504881544942E-2</v>
-      </c>
-      <c r="E68" s="8">
-        <v>0.37339455684646072</v>
-      </c>
-      <c r="F68" s="8">
-        <v>0.42321441056252979</v>
-      </c>
-      <c r="G68" s="8">
-        <v>0.18196029494668259</v>
-      </c>
-      <c r="H68" s="8">
-        <v>-5.8652325900180553E-2</v>
-      </c>
-      <c r="I68" s="8">
-        <v>-3.3938207838002832E-2</v>
-      </c>
-      <c r="J68" s="8">
-        <v>-5.446031360435577E-2</v>
-      </c>
-      <c r="K68" s="8">
-        <v>-9.2003360134670809E-2</v>
-      </c>
-      <c r="L68" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A69" s="7">
-        <v>4</v>
-      </c>
-      <c r="B69" s="8">
-        <v>0.33031034003778609</v>
-      </c>
-      <c r="C69" s="8">
-        <v>-0.2020297787671799</v>
-      </c>
-      <c r="D69" s="8">
-        <v>-6.9496230312799279E-2</v>
-      </c>
-      <c r="E69" s="8">
-        <v>0.45962118295891158</v>
-      </c>
-      <c r="F69" s="8">
-        <v>0.49560316311083918</v>
-      </c>
-      <c r="G69" s="8">
-        <v>0.29871273201842902</v>
-      </c>
-      <c r="H69" s="8">
-        <v>-9.9528700535100434E-2</v>
-      </c>
-      <c r="I69" s="8">
-        <v>-0.16550978323529919</v>
-      </c>
-      <c r="J69" s="8">
-        <v>-0.35211326660285103</v>
-      </c>
-      <c r="K69" s="8">
-        <v>-0.21086599623616389</v>
-      </c>
-      <c r="L69" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A70" s="4" t="s">
-        <v>280</v>
-      </c>
-      <c r="B70" s="8">
-        <v>0.40845973549716619</v>
-      </c>
-      <c r="C70" s="8">
-        <v>-0.22851485149413822</v>
-      </c>
-      <c r="D70" s="8">
-        <v>0.13961569356052095</v>
-      </c>
-      <c r="E70" s="8">
-        <v>0.4780866463891581</v>
-      </c>
-      <c r="F70" s="8">
-        <v>0.41283913785817761</v>
-      </c>
-      <c r="G70" s="8">
-        <v>0.49667331417674709</v>
-      </c>
-      <c r="H70" s="8">
-        <v>-6.4585829773739126E-2</v>
-      </c>
-      <c r="I70" s="8">
-        <v>-0.30841822468824392</v>
-      </c>
-      <c r="J70" s="8">
-        <v>-0.21568113252070359</v>
-      </c>
-      <c r="K70" s="8">
-        <v>-0.28072662168981544</v>
-      </c>
-      <c r="L70" s="8">
-        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>